<commit_message>
Currently able to plot R2 and RSME pairity plots for Tm and Hfus.
</commit_message>
<xml_diff>
--- a/data/input/MTGPR_Tm_Hfus_Hf/test_TBABH.xlsx
+++ b/data/input/MTGPR_Tm_Hfus_Hf/test_TBABH.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\aglotov\Eutectics\data\input\MTGPR_Tm_Hfus_Hf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FA48BA49-07B0-4402-B52B-11C9F19F4555}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05797EE2-8450-4799-B5DA-3D417987E584}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{535DD4A0-2912-47A9-820B-218FC7178EC0}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="7">
   <si>
     <t>T_m</t>
   </si>
@@ -53,10 +53,13 @@
     <t>SMILES</t>
   </si>
   <si>
-    <t>tetrabutylammonium borohydride</t>
-  </si>
-  <si>
-    <t>CCCC[N+](CCCC)(CCCC)CCCC.[BH4-]</t>
+    <t>ammonia borane</t>
+  </si>
+  <si>
+    <t>[BH3-][NH3+]</t>
+  </si>
+  <si>
+    <t>—</t>
   </si>
 </sst>
 </file>
@@ -428,14 +431,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB4AABDE-AFF5-4072-A990-39ABD46EABEB}">
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="42.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C1" t="s">
         <v>3</v>
       </c>
@@ -449,7 +452,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -457,10 +460,31 @@
         <v>5</v>
       </c>
       <c r="D2">
-        <v>402.15</v>
+        <v>384.15</v>
+      </c>
+      <c r="E2">
+        <v>9.8994949366116654</v>
+      </c>
+      <c r="F2">
+        <v>2</v>
       </c>
       <c r="G2">
-        <v>16.8</v>
+        <v>2.8</v>
+      </c>
+      <c r="H2">
+        <v>0.56568542494923979</v>
+      </c>
+      <c r="I2">
+        <v>2</v>
+      </c>
+      <c r="J2" t="s">
+        <v>6</v>
+      </c>
+      <c r="K2" t="s">
+        <v>6</v>
+      </c>
+      <c r="L2">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Created scripts to generate epoch and R^2 plots using a mixed model that learns the melting temperature and fusion "somewhat" seperately from the formation enthalpy.
</commit_message>
<xml_diff>
--- a/data/input/MTGPR_Tm_Hfus_Hf/test_TBABH.xlsx
+++ b/data/input/MTGPR_Tm_Hfus_Hf/test_TBABH.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\aglotov\Eutectics\data\input\MTGPR_Tm_Hfus_Hf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05797EE2-8450-4799-B5DA-3D417987E584}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2650DE7C-B9F7-4DB9-A36A-CBBA65F8649E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{535DD4A0-2912-47A9-820B-218FC7178EC0}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{535DD4A0-2912-47A9-820B-218FC7178EC0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="11">
   <si>
     <t>T_m</t>
   </si>
@@ -60,6 +60,18 @@
   </si>
   <si>
     <t>—</t>
+  </si>
+  <si>
+    <t>tetramethylammonium borohydride</t>
+  </si>
+  <si>
+    <t>tetrabutylammonium borohydride</t>
+  </si>
+  <si>
+    <t>[BH4-].CCCC[N+](CCCC)(CCCC)CCCC</t>
+  </si>
+  <si>
+    <t>[BH4-].C[N+](C)(C)C</t>
   </si>
 </sst>
 </file>
@@ -431,10 +443,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB4AABDE-AFF5-4072-A990-39ABD46EABEB}">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="31.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="42.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -487,6 +499,76 @@
         <v>0</v>
       </c>
     </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3">
+        <v>505.65</v>
+      </c>
+      <c r="E3">
+        <v>3.5355339059999999</v>
+      </c>
+      <c r="F3">
+        <v>2</v>
+      </c>
+      <c r="G3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H3" t="s">
+        <v>6</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3" t="s">
+        <v>6</v>
+      </c>
+      <c r="K3" t="s">
+        <v>6</v>
+      </c>
+      <c r="L3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4">
+        <v>402.15</v>
+      </c>
+      <c r="E4" t="s">
+        <v>6</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4">
+        <v>16.8</v>
+      </c>
+      <c r="H4">
+        <v>1.414213562</v>
+      </c>
+      <c r="I4">
+        <v>2</v>
+      </c>
+      <c r="J4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K4" t="s">
+        <v>6</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added Monte Carlo simulation for varying SLE conditions. Also tried more attempts at the MTGPR model.
</commit_message>
<xml_diff>
--- a/data/input/MTGPR_Tm_Hfus_Hf/test_TBABH.xlsx
+++ b/data/input/MTGPR_Tm_Hfus_Hf/test_TBABH.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\aglotov\Eutectics\data\input\MTGPR_Tm_Hfus_Hf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2650DE7C-B9F7-4DB9-A36A-CBBA65F8649E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{067DDF8B-F56A-4B8B-9A75-5729DE752FDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{535DD4A0-2912-47A9-820B-218FC7178EC0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{535DD4A0-2912-47A9-820B-218FC7178EC0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -56,9 +56,6 @@
     <t>ammonia borane</t>
   </si>
   <si>
-    <t>[BH3-][NH3+]</t>
-  </si>
-  <si>
     <t>—</t>
   </si>
   <si>
@@ -72,6 +69,9 @@
   </si>
   <si>
     <t>[BH4-].C[N+](C)(C)C</t>
+  </si>
+  <si>
+    <t>[B].N</t>
   </si>
 </sst>
 </file>
@@ -469,7 +469,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D2">
         <v>384.15</v>
@@ -490,10 +490,10 @@
         <v>2</v>
       </c>
       <c r="J2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L2">
         <v>0</v>
@@ -501,10 +501,10 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D3">
         <v>505.65</v>
@@ -516,19 +516,19 @@
         <v>2</v>
       </c>
       <c r="G3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I3">
         <v>0</v>
       </c>
       <c r="J3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L3">
         <v>0</v>
@@ -536,16 +536,16 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
         <v>8</v>
-      </c>
-      <c r="C4" t="s">
-        <v>9</v>
       </c>
       <c r="D4">
         <v>402.15</v>
       </c>
       <c r="E4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F4">
         <v>1</v>
@@ -560,10 +560,10 @@
         <v>2</v>
       </c>
       <c r="J4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L4">
         <v>0</v>

</xml_diff>

<commit_message>
Updated MTGPR model and obtained better results for ALL 3.
</commit_message>
<xml_diff>
--- a/data/input/MTGPR_Tm_Hfus_Hf/test_TBABH.xlsx
+++ b/data/input/MTGPR_Tm_Hfus_Hf/test_TBABH.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\aglotov\Eutectics\data\input\MTGPR_Tm_Hfus_Hf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{067DDF8B-F56A-4B8B-9A75-5729DE752FDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14E6820B-21EB-484C-A193-1B42A911496F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{535DD4A0-2912-47A9-820B-218FC7178EC0}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{535DD4A0-2912-47A9-820B-218FC7178EC0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="11">
   <si>
     <t>T_m</t>
   </si>
@@ -71,7 +71,7 @@
     <t>[BH4-].C[N+](C)(C)C</t>
   </si>
   <si>
-    <t>[B].N</t>
+    <t>B.N</t>
   </si>
 </sst>
 </file>
@@ -489,14 +489,14 @@
       <c r="I2">
         <v>2</v>
       </c>
-      <c r="J2" t="s">
-        <v>5</v>
+      <c r="J2">
+        <v>-133.4</v>
       </c>
       <c r="K2" t="s">
         <v>5</v>
       </c>
       <c r="L2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">

</xml_diff>